<commit_message>
Deploying to gh-pages from @ NavyaV4005/PawFeed2026@9821e5a7eb7509d8be8e6892c181838f68706776 🚀
</commit_message>
<xml_diff>
--- a/reports/selenium/selenium-test-results.xlsx
+++ b/reports/selenium/selenium-test-results.xlsx
@@ -30,7 +30,7 @@
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>7/27/2026, 8:21:42 AM</t>
+    <t>7/27/2026, 8:26:57 AM</t>
   </si>
   <si>
     <t>Total Tests Executed</t>
@@ -1074,7 +1074,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="2">
-        <v>2000</v>
+        <v>2089</v>
       </c>
     </row>
   </sheetData>
@@ -1325,7 +1325,7 @@
         <v>31</v>
       </c>
       <c r="D2" s="2">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>32</v>
@@ -1342,7 +1342,7 @@
         <v>31</v>
       </c>
       <c r="D3" s="2">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>32</v>
@@ -1359,7 +1359,7 @@
         <v>31</v>
       </c>
       <c r="D4" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>32</v>
@@ -1376,7 +1376,7 @@
         <v>31</v>
       </c>
       <c r="D5" s="2">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>32</v>
@@ -1393,7 +1393,7 @@
         <v>31</v>
       </c>
       <c r="D6" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>32</v>
@@ -1410,7 +1410,7 @@
         <v>31</v>
       </c>
       <c r="D7" s="2">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>32</v>
@@ -1427,7 +1427,7 @@
         <v>31</v>
       </c>
       <c r="D8" s="2">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>32</v>
@@ -1444,7 +1444,7 @@
         <v>31</v>
       </c>
       <c r="D9" s="2">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>32</v>
@@ -1461,7 +1461,7 @@
         <v>31</v>
       </c>
       <c r="D10" s="2">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>32</v>
@@ -1478,7 +1478,7 @@
         <v>31</v>
       </c>
       <c r="D11" s="2">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>32</v>
@@ -1495,7 +1495,7 @@
         <v>31</v>
       </c>
       <c r="D12" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>32</v>
@@ -1512,7 +1512,7 @@
         <v>31</v>
       </c>
       <c r="D13" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>32</v>
@@ -1529,7 +1529,7 @@
         <v>31</v>
       </c>
       <c r="D14" s="2">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>32</v>
@@ -1546,7 +1546,7 @@
         <v>31</v>
       </c>
       <c r="D15" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>32</v>
@@ -1563,7 +1563,7 @@
         <v>31</v>
       </c>
       <c r="D16" s="2">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>32</v>
@@ -1580,7 +1580,7 @@
         <v>31</v>
       </c>
       <c r="D17" s="2">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>32</v>
@@ -1597,7 +1597,7 @@
         <v>31</v>
       </c>
       <c r="D18" s="2">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>32</v>
@@ -1614,7 +1614,7 @@
         <v>31</v>
       </c>
       <c r="D19" s="2">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>32</v>
@@ -1631,7 +1631,7 @@
         <v>31</v>
       </c>
       <c r="D20" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>32</v>
@@ -1648,7 +1648,7 @@
         <v>31</v>
       </c>
       <c r="D21" s="2">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>32</v>
@@ -1665,7 +1665,7 @@
         <v>31</v>
       </c>
       <c r="D22" s="2">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>32</v>
@@ -1682,7 +1682,7 @@
         <v>31</v>
       </c>
       <c r="D23" s="2">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>32</v>
@@ -1699,7 +1699,7 @@
         <v>31</v>
       </c>
       <c r="D24" s="2">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>32</v>
@@ -1716,7 +1716,7 @@
         <v>31</v>
       </c>
       <c r="D25" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>32</v>
@@ -1733,7 +1733,7 @@
         <v>31</v>
       </c>
       <c r="D26" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>32</v>
@@ -1750,7 +1750,7 @@
         <v>31</v>
       </c>
       <c r="D27" s="2">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>32</v>
@@ -1767,7 +1767,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>32</v>
@@ -1784,7 +1784,7 @@
         <v>31</v>
       </c>
       <c r="D29" s="2">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>32</v>
@@ -1801,7 +1801,7 @@
         <v>31</v>
       </c>
       <c r="D30" s="2">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>32</v>
@@ -1818,7 +1818,7 @@
         <v>31</v>
       </c>
       <c r="D31" s="2">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>32</v>
@@ -1852,7 +1852,7 @@
         <v>31</v>
       </c>
       <c r="D33" s="2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>32</v>
@@ -1869,7 +1869,7 @@
         <v>31</v>
       </c>
       <c r="D34" s="2">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>32</v>
@@ -1886,7 +1886,7 @@
         <v>31</v>
       </c>
       <c r="D35" s="2">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>32</v>
@@ -1903,7 +1903,7 @@
         <v>31</v>
       </c>
       <c r="D36" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>32</v>
@@ -1920,7 +1920,7 @@
         <v>31</v>
       </c>
       <c r="D37" s="2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>32</v>
@@ -1937,7 +1937,7 @@
         <v>31</v>
       </c>
       <c r="D38" s="2">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>32</v>
@@ -1971,7 +1971,7 @@
         <v>31</v>
       </c>
       <c r="D40" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>32</v>
@@ -1988,7 +1988,7 @@
         <v>31</v>
       </c>
       <c r="D41" s="2">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>32</v>
@@ -2005,7 +2005,7 @@
         <v>31</v>
       </c>
       <c r="D42" s="2">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>32</v>
@@ -2022,7 +2022,7 @@
         <v>31</v>
       </c>
       <c r="D43" s="2">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>32</v>
@@ -2039,7 +2039,7 @@
         <v>31</v>
       </c>
       <c r="D44" s="2">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>32</v>
@@ -2056,7 +2056,7 @@
         <v>31</v>
       </c>
       <c r="D45" s="2">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>32</v>
@@ -2073,7 +2073,7 @@
         <v>31</v>
       </c>
       <c r="D46" s="2">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>32</v>
@@ -2090,7 +2090,7 @@
         <v>31</v>
       </c>
       <c r="D47" s="2">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>32</v>
@@ -2107,7 +2107,7 @@
         <v>31</v>
       </c>
       <c r="D48" s="2">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>32</v>
@@ -2158,7 +2158,7 @@
         <v>31</v>
       </c>
       <c r="D51" s="2">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>32</v>
@@ -2175,7 +2175,7 @@
         <v>31</v>
       </c>
       <c r="D52" s="2">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>32</v>
@@ -2192,7 +2192,7 @@
         <v>31</v>
       </c>
       <c r="D53" s="2">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>32</v>
@@ -2209,7 +2209,7 @@
         <v>31</v>
       </c>
       <c r="D54" s="2">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>32</v>
@@ -2243,7 +2243,7 @@
         <v>31</v>
       </c>
       <c r="D56" s="2">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>32</v>
@@ -2260,7 +2260,7 @@
         <v>31</v>
       </c>
       <c r="D57" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>32</v>
@@ -2277,7 +2277,7 @@
         <v>31</v>
       </c>
       <c r="D58" s="2">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>32</v>
@@ -2294,7 +2294,7 @@
         <v>31</v>
       </c>
       <c r="D59" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>32</v>
@@ -2311,7 +2311,7 @@
         <v>31</v>
       </c>
       <c r="D60" s="2">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>32</v>
@@ -2328,7 +2328,7 @@
         <v>31</v>
       </c>
       <c r="D61" s="2">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>32</v>
@@ -2345,7 +2345,7 @@
         <v>31</v>
       </c>
       <c r="D62" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>32</v>
@@ -2362,7 +2362,7 @@
         <v>31</v>
       </c>
       <c r="D63" s="2">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>32</v>
@@ -2379,7 +2379,7 @@
         <v>31</v>
       </c>
       <c r="D64" s="2">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>32</v>
@@ -2396,7 +2396,7 @@
         <v>31</v>
       </c>
       <c r="D65" s="2">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>32</v>
@@ -2413,7 +2413,7 @@
         <v>31</v>
       </c>
       <c r="D66" s="2">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>32</v>
@@ -2430,7 +2430,7 @@
         <v>31</v>
       </c>
       <c r="D67" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>32</v>
@@ -2447,7 +2447,7 @@
         <v>31</v>
       </c>
       <c r="D68" s="2">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>32</v>
@@ -2464,7 +2464,7 @@
         <v>31</v>
       </c>
       <c r="D69" s="2">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>32</v>
@@ -2481,7 +2481,7 @@
         <v>31</v>
       </c>
       <c r="D70" s="2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>32</v>
@@ -2498,7 +2498,7 @@
         <v>31</v>
       </c>
       <c r="D71" s="2">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>32</v>
@@ -2515,7 +2515,7 @@
         <v>31</v>
       </c>
       <c r="D72" s="2">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>32</v>
@@ -2532,7 +2532,7 @@
         <v>31</v>
       </c>
       <c r="D73" s="2">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>32</v>
@@ -2549,7 +2549,7 @@
         <v>31</v>
       </c>
       <c r="D74" s="2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>32</v>
@@ -2566,7 +2566,7 @@
         <v>31</v>
       </c>
       <c r="D75" s="2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>32</v>
@@ -2583,7 +2583,7 @@
         <v>31</v>
       </c>
       <c r="D76" s="2">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>32</v>
@@ -2600,7 +2600,7 @@
         <v>31</v>
       </c>
       <c r="D77" s="2">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>32</v>
@@ -2617,7 +2617,7 @@
         <v>31</v>
       </c>
       <c r="D78" s="2">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>32</v>
@@ -2634,7 +2634,7 @@
         <v>31</v>
       </c>
       <c r="D79" s="2">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>32</v>
@@ -2651,7 +2651,7 @@
         <v>31</v>
       </c>
       <c r="D80" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>32</v>
@@ -2668,7 +2668,7 @@
         <v>31</v>
       </c>
       <c r="D81" s="2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>32</v>
@@ -2685,7 +2685,7 @@
         <v>31</v>
       </c>
       <c r="D82" s="2">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>32</v>
@@ -2702,7 +2702,7 @@
         <v>31</v>
       </c>
       <c r="D83" s="2">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>32</v>
@@ -2719,7 +2719,7 @@
         <v>31</v>
       </c>
       <c r="D84" s="2">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>32</v>
@@ -2736,7 +2736,7 @@
         <v>31</v>
       </c>
       <c r="D85" s="2">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>32</v>
@@ -2753,7 +2753,7 @@
         <v>31</v>
       </c>
       <c r="D86" s="2">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>32</v>
@@ -2770,7 +2770,7 @@
         <v>31</v>
       </c>
       <c r="D87" s="2">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>32</v>
@@ -2804,7 +2804,7 @@
         <v>31</v>
       </c>
       <c r="D89" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>32</v>
@@ -2821,7 +2821,7 @@
         <v>31</v>
       </c>
       <c r="D90" s="2">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>32</v>
@@ -2838,7 +2838,7 @@
         <v>31</v>
       </c>
       <c r="D91" s="2">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>32</v>
@@ -2855,7 +2855,7 @@
         <v>31</v>
       </c>
       <c r="D92" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>32</v>
@@ -2872,7 +2872,7 @@
         <v>31</v>
       </c>
       <c r="D93" s="2">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>32</v>
@@ -2889,7 +2889,7 @@
         <v>31</v>
       </c>
       <c r="D94" s="2">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>32</v>
@@ -2906,7 +2906,7 @@
         <v>31</v>
       </c>
       <c r="D95" s="2">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>32</v>
@@ -2923,7 +2923,7 @@
         <v>31</v>
       </c>
       <c r="D96" s="2">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>32</v>
@@ -2940,7 +2940,7 @@
         <v>31</v>
       </c>
       <c r="D97" s="2">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>32</v>
@@ -2957,7 +2957,7 @@
         <v>31</v>
       </c>
       <c r="D98" s="2">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>32</v>
@@ -2974,7 +2974,7 @@
         <v>31</v>
       </c>
       <c r="D99" s="2">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>32</v>
@@ -2991,7 +2991,7 @@
         <v>31</v>
       </c>
       <c r="D100" s="2">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>32</v>
@@ -3008,7 +3008,7 @@
         <v>31</v>
       </c>
       <c r="D101" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>32</v>
@@ -3025,7 +3025,7 @@
         <v>31</v>
       </c>
       <c r="D102" s="2">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>32</v>
@@ -3042,7 +3042,7 @@
         <v>31</v>
       </c>
       <c r="D103" s="2">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>32</v>
@@ -3059,7 +3059,7 @@
         <v>31</v>
       </c>
       <c r="D104" s="2">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E104" s="2" t="s">
         <v>32</v>
@@ -3076,7 +3076,7 @@
         <v>31</v>
       </c>
       <c r="D105" s="2">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>32</v>
@@ -3093,7 +3093,7 @@
         <v>31</v>
       </c>
       <c r="D106" s="2">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>32</v>
@@ -3110,7 +3110,7 @@
         <v>31</v>
       </c>
       <c r="D107" s="2">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>32</v>
@@ -3127,7 +3127,7 @@
         <v>31</v>
       </c>
       <c r="D108" s="2">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>32</v>
@@ -3144,7 +3144,7 @@
         <v>31</v>
       </c>
       <c r="D109" s="2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>32</v>
@@ -3161,7 +3161,7 @@
         <v>31</v>
       </c>
       <c r="D110" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>32</v>
@@ -3178,7 +3178,7 @@
         <v>31</v>
       </c>
       <c r="D111" s="2">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>32</v>
@@ -3195,7 +3195,7 @@
         <v>31</v>
       </c>
       <c r="D112" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>32</v>
@@ -3212,7 +3212,7 @@
         <v>31</v>
       </c>
       <c r="D113" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>32</v>
@@ -3229,7 +3229,7 @@
         <v>31</v>
       </c>
       <c r="D114" s="2">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>32</v>
@@ -3246,7 +3246,7 @@
         <v>31</v>
       </c>
       <c r="D115" s="2">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>32</v>
@@ -3263,7 +3263,7 @@
         <v>31</v>
       </c>
       <c r="D116" s="2">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E116" s="2" t="s">
         <v>32</v>
@@ -3280,7 +3280,7 @@
         <v>31</v>
       </c>
       <c r="D117" s="2">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>32</v>
@@ -3297,7 +3297,7 @@
         <v>31</v>
       </c>
       <c r="D118" s="2">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>32</v>
@@ -3314,7 +3314,7 @@
         <v>31</v>
       </c>
       <c r="D119" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E119" s="2" t="s">
         <v>32</v>
@@ -3331,7 +3331,7 @@
         <v>31</v>
       </c>
       <c r="D120" s="2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E120" s="2" t="s">
         <v>32</v>
@@ -3348,7 +3348,7 @@
         <v>31</v>
       </c>
       <c r="D121" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E121" s="2" t="s">
         <v>32</v>
@@ -3365,7 +3365,7 @@
         <v>31</v>
       </c>
       <c r="D122" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E122" s="2" t="s">
         <v>32</v>
@@ -3382,7 +3382,7 @@
         <v>31</v>
       </c>
       <c r="D123" s="2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>32</v>
@@ -3399,7 +3399,7 @@
         <v>31</v>
       </c>
       <c r="D124" s="2">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>32</v>
@@ -3416,7 +3416,7 @@
         <v>31</v>
       </c>
       <c r="D125" s="2">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>32</v>
@@ -3433,7 +3433,7 @@
         <v>31</v>
       </c>
       <c r="D126" s="2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>32</v>
@@ -3450,7 +3450,7 @@
         <v>31</v>
       </c>
       <c r="D127" s="2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>32</v>
@@ -3467,7 +3467,7 @@
         <v>31</v>
       </c>
       <c r="D128" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>32</v>
@@ -3484,7 +3484,7 @@
         <v>31</v>
       </c>
       <c r="D129" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>32</v>
@@ -3501,7 +3501,7 @@
         <v>31</v>
       </c>
       <c r="D130" s="2">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>32</v>
@@ -3518,7 +3518,7 @@
         <v>31</v>
       </c>
       <c r="D131" s="2">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>32</v>
@@ -3535,7 +3535,7 @@
         <v>31</v>
       </c>
       <c r="D132" s="2">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>32</v>
@@ -3552,7 +3552,7 @@
         <v>31</v>
       </c>
       <c r="D133" s="2">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>32</v>
@@ -3569,7 +3569,7 @@
         <v>31</v>
       </c>
       <c r="D134" s="2">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>32</v>
@@ -3586,7 +3586,7 @@
         <v>31</v>
       </c>
       <c r="D135" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>32</v>
@@ -3603,7 +3603,7 @@
         <v>31</v>
       </c>
       <c r="D136" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>32</v>
@@ -3620,7 +3620,7 @@
         <v>31</v>
       </c>
       <c r="D137" s="2">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>32</v>
@@ -3637,7 +3637,7 @@
         <v>31</v>
       </c>
       <c r="D138" s="2">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>32</v>
@@ -3654,7 +3654,7 @@
         <v>31</v>
       </c>
       <c r="D139" s="2">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>32</v>
@@ -3671,7 +3671,7 @@
         <v>31</v>
       </c>
       <c r="D140" s="2">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>32</v>
@@ -3688,7 +3688,7 @@
         <v>31</v>
       </c>
       <c r="D141" s="2">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>32</v>
@@ -3705,7 +3705,7 @@
         <v>31</v>
       </c>
       <c r="D142" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>32</v>
@@ -3722,7 +3722,7 @@
         <v>31</v>
       </c>
       <c r="D143" s="2">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>32</v>
@@ -3756,7 +3756,7 @@
         <v>31</v>
       </c>
       <c r="D145" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>32</v>
@@ -3773,7 +3773,7 @@
         <v>31</v>
       </c>
       <c r="D146" s="2">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E146" s="2" t="s">
         <v>32</v>
@@ -3790,7 +3790,7 @@
         <v>31</v>
       </c>
       <c r="D147" s="2">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>32</v>
@@ -3807,7 +3807,7 @@
         <v>31</v>
       </c>
       <c r="D148" s="2">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E148" s="2" t="s">
         <v>32</v>
@@ -3824,7 +3824,7 @@
         <v>31</v>
       </c>
       <c r="D149" s="2">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>32</v>
@@ -3841,7 +3841,7 @@
         <v>31</v>
       </c>
       <c r="D150" s="2">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E150" s="2" t="s">
         <v>32</v>
@@ -3858,7 +3858,7 @@
         <v>31</v>
       </c>
       <c r="D151" s="2">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E151" s="2" t="s">
         <v>32</v>
@@ -3875,7 +3875,7 @@
         <v>31</v>
       </c>
       <c r="D152" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E152" s="2" t="s">
         <v>32</v>
@@ -3892,7 +3892,7 @@
         <v>31</v>
       </c>
       <c r="D153" s="2">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E153" s="2" t="s">
         <v>32</v>
@@ -3909,7 +3909,7 @@
         <v>31</v>
       </c>
       <c r="D154" s="2">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E154" s="2" t="s">
         <v>32</v>
@@ -3926,7 +3926,7 @@
         <v>31</v>
       </c>
       <c r="D155" s="2">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E155" s="2" t="s">
         <v>32</v>
@@ -3943,7 +3943,7 @@
         <v>31</v>
       </c>
       <c r="D156" s="2">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E156" s="2" t="s">
         <v>32</v>
@@ -3960,7 +3960,7 @@
         <v>31</v>
       </c>
       <c r="D157" s="2">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E157" s="2" t="s">
         <v>32</v>
@@ -3977,7 +3977,7 @@
         <v>31</v>
       </c>
       <c r="D158" s="2">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E158" s="2" t="s">
         <v>32</v>
@@ -3994,7 +3994,7 @@
         <v>31</v>
       </c>
       <c r="D159" s="2">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E159" s="2" t="s">
         <v>32</v>
@@ -4011,7 +4011,7 @@
         <v>31</v>
       </c>
       <c r="D160" s="2">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E160" s="2" t="s">
         <v>32</v>
@@ -4028,7 +4028,7 @@
         <v>31</v>
       </c>
       <c r="D161" s="2">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E161" s="2" t="s">
         <v>32</v>

</xml_diff>